<commit_message>
Integra ubigeo_cui y ubigeo_pronied: departamento al 100%
- ubigeo_cui.csv: enriquecimiento geografico por CUI (364,230 CUI), rescata
  registros cuyo cod_local no figura en los padrones (Grupo 2 PI baja de 191 a
  32 sin departamento).
- ubigeo_pronied.xlsx: fuente adicional cod_local -> geo (DRE/UGEL, nombre IE,
  ruralidad) y cod_mod -> cod_local. Area normalizada a Urbana/Rural.
- Fusion de todas las fuentes a nivel de campo (sin sobrescribir lo conocido).
- Cobertura final: departamento 100%, DRE 99.9%, UGEL 99.7%, area 99.6%.

https://claude.ai/code/session_01N9afypBcQVKYhttom8P34Z
</commit_message>
<xml_diff>
--- a/output/bases_limpias/Grupo_01_MOBILIARIO_Y_EQUIPO/df_drelm_mobiliario.xlsx
+++ b/output/bases_limpias/Grupo_01_MOBILIARIO_Y_EQUIPO/df_drelm_mobiliario.xlsx
@@ -7689,7 +7689,11 @@
           <t>VILLA EL SALVADOR</t>
         </is>
       </c>
-      <c r="K87" t="inlineStr"/>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>VILLA EL SALVADOR</t>
+        </is>
+      </c>
       <c r="L87" t="inlineStr">
         <is>
           <t>150142</t>

</xml_diff>